<commit_message>
feat: add bundle-parsing ingestion script, correct data dictionary field paths
</commit_message>
<xml_diff>
--- a/docs/data_dictionary.xlsx
+++ b/docs/data_dictionary.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Tables" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staging Models" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intermediate Models" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mart Models" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBP Measure Logic" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contract Terms" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Raw Tables" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Staging Models" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Intermediate Models" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Mart Models" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CBP Measure Logic" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Contract Terms" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -778,7 +778,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>id, subject.reference, code (JSON), value, effectiveDateTime</t>
+          <t>id, subject.reference, code (JSON, panel-level e.g. 85354-9), component (JSON array - actual BP systolic/diastolic values live here, NOT a top-level value field), effectiveDateTime</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -791,7 +791,11 @@
           <t>Planned</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr"/>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>BP values are nested in component[]; component[].code.coding[].code identifies systolic (8480-6) vs diastolic (8462-4)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -811,7 +815,7 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>id, patient.reference, billablePeriod, item (JSON)</t>
+          <t>id, patient.reference, billablePeriod, total (JSON), item (JSON)</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -844,7 +848,7 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>id, patient.reference, payment (JSON), item (JSON)</t>
+          <t>id, patient.reference, payment (JSON, actual paid amount), total (JSON array, categorized by adjudication type), item (JSON)</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -857,7 +861,11 @@
           <t>Planned</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>total is an array keyed by total[].category.coding[].code (e.g. Submitted Amount) - not a single total; payment.amount.value is the actual paid amount</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -1057,7 +1065,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Resolve patient_id; extract code, value (numeric or coded), unit</t>
+          <t>Resolve patient_id; unnest component[] array to get systolic/diastolic as separate columns (join on component.code.coding.code = 8480-6 / 8462-4); extract effectiveDateTime</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -1070,7 +1078,11 @@
           <t>Planned</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>BP panel resources have no top-level value - must unnest component[]</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -1085,7 +1097,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Resolve patient_id; extract billable period, line items</t>
+          <t>Resolve patient_id; extract billable period, total.value, line items</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -1113,7 +1125,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Resolve patient_id; extract allowed/paid amounts</t>
+          <t>Resolve patient_id; extract payment.amount.value (actual paid); filter total[] by category code for submitted/allowed amounts</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -1126,7 +1138,11 @@
           <t>Planned</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>total[] is categorized by adjudication type, not a single amount</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">

</xml_diff>